<commit_message>
Fix the malformed action formulas in the betting workbook
Each of the six recommendation columns opened five IF( calls but closed six
times, so Excel treated the workbook as corrupt, offered to repair it, and
stripped every one of those cells. The spread, moneyline and total action
columns on both the Bets and Live sheets loaded blank, which is the one output
of the report a user acts on.

Drop the stray parenthesis and validate the generated workbook by tokenizing
every formula rather than counting characters, so nesting that balances overall
but closes too early is caught as well. The Bets sheet now emits 624 formulas
where it previously emitted 576.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/week_01_2026_betting.xlsx
+++ b/reports/week_01_2026_betting.xlsx
@@ -1164,7 +1164,7 @@
         <v/>
       </c>
       <c r="AR2">
-        <f>IF(AQ2&lt;=0,"PASS",IF(AQ2&lt;0.02,"PASS",IF(AQ2&lt;0.04,"LEAN",IF(AQ2&lt;0.07,"SMALL",IF(AQ2&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ2&lt;=0,"PASS",IF(AQ2&lt;0.02,"PASS",IF(AQ2&lt;0.04,"LEAN",IF(AQ2&lt;0.07,"SMALL",IF(AQ2&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS2" s="4">
@@ -1184,7 +1184,7 @@
         <v/>
       </c>
       <c r="AW2">
-        <f>IF(AV2&lt;=0,"PASS",IF(AV2&lt;0.02,"PASS",IF(AV2&lt;0.04,"LEAN",IF(AV2&lt;0.07,"SMALL",IF(AV2&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV2&lt;=0,"PASS",IF(AV2&lt;0.02,"PASS",IF(AV2&lt;0.04,"LEAN",IF(AV2&lt;0.07,"SMALL",IF(AV2&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX2" s="4">
@@ -1204,7 +1204,7 @@
         <v/>
       </c>
       <c r="BB2">
-        <f>IF(BA2&lt;=0,"PASS",IF(BA2&lt;0.02,"PASS",IF(BA2&lt;0.04,"LEAN",IF(BA2&lt;0.07,"SMALL",IF(BA2&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA2&lt;=0,"PASS",IF(BA2&lt;0.02,"PASS",IF(BA2&lt;0.04,"LEAN",IF(BA2&lt;0.07,"SMALL",IF(BA2&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC2" s="4">
@@ -1431,7 +1431,7 @@
         <v/>
       </c>
       <c r="AR3">
-        <f>IF(AQ3&lt;=0,"PASS",IF(AQ3&lt;0.02,"PASS",IF(AQ3&lt;0.04,"LEAN",IF(AQ3&lt;0.07,"SMALL",IF(AQ3&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ3&lt;=0,"PASS",IF(AQ3&lt;0.02,"PASS",IF(AQ3&lt;0.04,"LEAN",IF(AQ3&lt;0.07,"SMALL",IF(AQ3&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS3" s="4">
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="AW3">
-        <f>IF(AV3&lt;=0,"PASS",IF(AV3&lt;0.02,"PASS",IF(AV3&lt;0.04,"LEAN",IF(AV3&lt;0.07,"SMALL",IF(AV3&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV3&lt;=0,"PASS",IF(AV3&lt;0.02,"PASS",IF(AV3&lt;0.04,"LEAN",IF(AV3&lt;0.07,"SMALL",IF(AV3&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX3" s="4">
@@ -1471,7 +1471,7 @@
         <v/>
       </c>
       <c r="BB3">
-        <f>IF(BA3&lt;=0,"PASS",IF(BA3&lt;0.02,"PASS",IF(BA3&lt;0.04,"LEAN",IF(BA3&lt;0.07,"SMALL",IF(BA3&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA3&lt;=0,"PASS",IF(BA3&lt;0.02,"PASS",IF(BA3&lt;0.04,"LEAN",IF(BA3&lt;0.07,"SMALL",IF(BA3&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC3" s="4">
@@ -1698,7 +1698,7 @@
         <v/>
       </c>
       <c r="AR4">
-        <f>IF(AQ4&lt;=0,"PASS",IF(AQ4&lt;0.02,"PASS",IF(AQ4&lt;0.04,"LEAN",IF(AQ4&lt;0.07,"SMALL",IF(AQ4&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ4&lt;=0,"PASS",IF(AQ4&lt;0.02,"PASS",IF(AQ4&lt;0.04,"LEAN",IF(AQ4&lt;0.07,"SMALL",IF(AQ4&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS4" s="4">
@@ -1718,7 +1718,7 @@
         <v/>
       </c>
       <c r="AW4">
-        <f>IF(AV4&lt;=0,"PASS",IF(AV4&lt;0.02,"PASS",IF(AV4&lt;0.04,"LEAN",IF(AV4&lt;0.07,"SMALL",IF(AV4&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV4&lt;=0,"PASS",IF(AV4&lt;0.02,"PASS",IF(AV4&lt;0.04,"LEAN",IF(AV4&lt;0.07,"SMALL",IF(AV4&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX4" s="4">
@@ -1738,7 +1738,7 @@
         <v/>
       </c>
       <c r="BB4">
-        <f>IF(BA4&lt;=0,"PASS",IF(BA4&lt;0.02,"PASS",IF(BA4&lt;0.04,"LEAN",IF(BA4&lt;0.07,"SMALL",IF(BA4&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA4&lt;=0,"PASS",IF(BA4&lt;0.02,"PASS",IF(BA4&lt;0.04,"LEAN",IF(BA4&lt;0.07,"SMALL",IF(BA4&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC4" s="4">
@@ -1965,7 +1965,7 @@
         <v/>
       </c>
       <c r="AR5">
-        <f>IF(AQ5&lt;=0,"PASS",IF(AQ5&lt;0.02,"PASS",IF(AQ5&lt;0.04,"LEAN",IF(AQ5&lt;0.07,"SMALL",IF(AQ5&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ5&lt;=0,"PASS",IF(AQ5&lt;0.02,"PASS",IF(AQ5&lt;0.04,"LEAN",IF(AQ5&lt;0.07,"SMALL",IF(AQ5&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS5" s="4">
@@ -1985,7 +1985,7 @@
         <v/>
       </c>
       <c r="AW5">
-        <f>IF(AV5&lt;=0,"PASS",IF(AV5&lt;0.02,"PASS",IF(AV5&lt;0.04,"LEAN",IF(AV5&lt;0.07,"SMALL",IF(AV5&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV5&lt;=0,"PASS",IF(AV5&lt;0.02,"PASS",IF(AV5&lt;0.04,"LEAN",IF(AV5&lt;0.07,"SMALL",IF(AV5&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX5" s="4">
@@ -2005,7 +2005,7 @@
         <v/>
       </c>
       <c r="BB5">
-        <f>IF(BA5&lt;=0,"PASS",IF(BA5&lt;0.02,"PASS",IF(BA5&lt;0.04,"LEAN",IF(BA5&lt;0.07,"SMALL",IF(BA5&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA5&lt;=0,"PASS",IF(BA5&lt;0.02,"PASS",IF(BA5&lt;0.04,"LEAN",IF(BA5&lt;0.07,"SMALL",IF(BA5&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC5" s="4">
@@ -2232,7 +2232,7 @@
         <v/>
       </c>
       <c r="AR6">
-        <f>IF(AQ6&lt;=0,"PASS",IF(AQ6&lt;0.02,"PASS",IF(AQ6&lt;0.04,"LEAN",IF(AQ6&lt;0.07,"SMALL",IF(AQ6&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ6&lt;=0,"PASS",IF(AQ6&lt;0.02,"PASS",IF(AQ6&lt;0.04,"LEAN",IF(AQ6&lt;0.07,"SMALL",IF(AQ6&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS6" s="4">
@@ -2252,7 +2252,7 @@
         <v/>
       </c>
       <c r="AW6">
-        <f>IF(AV6&lt;=0,"PASS",IF(AV6&lt;0.02,"PASS",IF(AV6&lt;0.04,"LEAN",IF(AV6&lt;0.07,"SMALL",IF(AV6&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV6&lt;=0,"PASS",IF(AV6&lt;0.02,"PASS",IF(AV6&lt;0.04,"LEAN",IF(AV6&lt;0.07,"SMALL",IF(AV6&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX6" s="4">
@@ -2272,7 +2272,7 @@
         <v/>
       </c>
       <c r="BB6">
-        <f>IF(BA6&lt;=0,"PASS",IF(BA6&lt;0.02,"PASS",IF(BA6&lt;0.04,"LEAN",IF(BA6&lt;0.07,"SMALL",IF(BA6&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA6&lt;=0,"PASS",IF(BA6&lt;0.02,"PASS",IF(BA6&lt;0.04,"LEAN",IF(BA6&lt;0.07,"SMALL",IF(BA6&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC6" s="4">
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="AR7">
-        <f>IF(AQ7&lt;=0,"PASS",IF(AQ7&lt;0.02,"PASS",IF(AQ7&lt;0.04,"LEAN",IF(AQ7&lt;0.07,"SMALL",IF(AQ7&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ7&lt;=0,"PASS",IF(AQ7&lt;0.02,"PASS",IF(AQ7&lt;0.04,"LEAN",IF(AQ7&lt;0.07,"SMALL",IF(AQ7&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS7" s="4">
@@ -2519,7 +2519,7 @@
         <v/>
       </c>
       <c r="AW7">
-        <f>IF(AV7&lt;=0,"PASS",IF(AV7&lt;0.02,"PASS",IF(AV7&lt;0.04,"LEAN",IF(AV7&lt;0.07,"SMALL",IF(AV7&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV7&lt;=0,"PASS",IF(AV7&lt;0.02,"PASS",IF(AV7&lt;0.04,"LEAN",IF(AV7&lt;0.07,"SMALL",IF(AV7&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX7" s="4">
@@ -2539,7 +2539,7 @@
         <v/>
       </c>
       <c r="BB7">
-        <f>IF(BA7&lt;=0,"PASS",IF(BA7&lt;0.02,"PASS",IF(BA7&lt;0.04,"LEAN",IF(BA7&lt;0.07,"SMALL",IF(BA7&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA7&lt;=0,"PASS",IF(BA7&lt;0.02,"PASS",IF(BA7&lt;0.04,"LEAN",IF(BA7&lt;0.07,"SMALL",IF(BA7&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC7" s="4">
@@ -2766,7 +2766,7 @@
         <v/>
       </c>
       <c r="AR8">
-        <f>IF(AQ8&lt;=0,"PASS",IF(AQ8&lt;0.02,"PASS",IF(AQ8&lt;0.04,"LEAN",IF(AQ8&lt;0.07,"SMALL",IF(AQ8&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ8&lt;=0,"PASS",IF(AQ8&lt;0.02,"PASS",IF(AQ8&lt;0.04,"LEAN",IF(AQ8&lt;0.07,"SMALL",IF(AQ8&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS8" s="4">
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="AW8">
-        <f>IF(AV8&lt;=0,"PASS",IF(AV8&lt;0.02,"PASS",IF(AV8&lt;0.04,"LEAN",IF(AV8&lt;0.07,"SMALL",IF(AV8&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV8&lt;=0,"PASS",IF(AV8&lt;0.02,"PASS",IF(AV8&lt;0.04,"LEAN",IF(AV8&lt;0.07,"SMALL",IF(AV8&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX8" s="4">
@@ -2806,7 +2806,7 @@
         <v/>
       </c>
       <c r="BB8">
-        <f>IF(BA8&lt;=0,"PASS",IF(BA8&lt;0.02,"PASS",IF(BA8&lt;0.04,"LEAN",IF(BA8&lt;0.07,"SMALL",IF(BA8&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA8&lt;=0,"PASS",IF(BA8&lt;0.02,"PASS",IF(BA8&lt;0.04,"LEAN",IF(BA8&lt;0.07,"SMALL",IF(BA8&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC8" s="4">
@@ -3033,7 +3033,7 @@
         <v/>
       </c>
       <c r="AR9">
-        <f>IF(AQ9&lt;=0,"PASS",IF(AQ9&lt;0.02,"PASS",IF(AQ9&lt;0.04,"LEAN",IF(AQ9&lt;0.07,"SMALL",IF(AQ9&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ9&lt;=0,"PASS",IF(AQ9&lt;0.02,"PASS",IF(AQ9&lt;0.04,"LEAN",IF(AQ9&lt;0.07,"SMALL",IF(AQ9&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS9" s="4">
@@ -3053,7 +3053,7 @@
         <v/>
       </c>
       <c r="AW9">
-        <f>IF(AV9&lt;=0,"PASS",IF(AV9&lt;0.02,"PASS",IF(AV9&lt;0.04,"LEAN",IF(AV9&lt;0.07,"SMALL",IF(AV9&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV9&lt;=0,"PASS",IF(AV9&lt;0.02,"PASS",IF(AV9&lt;0.04,"LEAN",IF(AV9&lt;0.07,"SMALL",IF(AV9&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX9" s="4">
@@ -3073,7 +3073,7 @@
         <v/>
       </c>
       <c r="BB9">
-        <f>IF(BA9&lt;=0,"PASS",IF(BA9&lt;0.02,"PASS",IF(BA9&lt;0.04,"LEAN",IF(BA9&lt;0.07,"SMALL",IF(BA9&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA9&lt;=0,"PASS",IF(BA9&lt;0.02,"PASS",IF(BA9&lt;0.04,"LEAN",IF(BA9&lt;0.07,"SMALL",IF(BA9&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC9" s="4">
@@ -3300,7 +3300,7 @@
         <v/>
       </c>
       <c r="AR10">
-        <f>IF(AQ10&lt;=0,"PASS",IF(AQ10&lt;0.02,"PASS",IF(AQ10&lt;0.04,"LEAN",IF(AQ10&lt;0.07,"SMALL",IF(AQ10&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ10&lt;=0,"PASS",IF(AQ10&lt;0.02,"PASS",IF(AQ10&lt;0.04,"LEAN",IF(AQ10&lt;0.07,"SMALL",IF(AQ10&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS10" s="4">
@@ -3320,7 +3320,7 @@
         <v/>
       </c>
       <c r="AW10">
-        <f>IF(AV10&lt;=0,"PASS",IF(AV10&lt;0.02,"PASS",IF(AV10&lt;0.04,"LEAN",IF(AV10&lt;0.07,"SMALL",IF(AV10&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV10&lt;=0,"PASS",IF(AV10&lt;0.02,"PASS",IF(AV10&lt;0.04,"LEAN",IF(AV10&lt;0.07,"SMALL",IF(AV10&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX10" s="4">
@@ -3340,7 +3340,7 @@
         <v/>
       </c>
       <c r="BB10">
-        <f>IF(BA10&lt;=0,"PASS",IF(BA10&lt;0.02,"PASS",IF(BA10&lt;0.04,"LEAN",IF(BA10&lt;0.07,"SMALL",IF(BA10&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA10&lt;=0,"PASS",IF(BA10&lt;0.02,"PASS",IF(BA10&lt;0.04,"LEAN",IF(BA10&lt;0.07,"SMALL",IF(BA10&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC10" s="4">
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AR11">
-        <f>IF(AQ11&lt;=0,"PASS",IF(AQ11&lt;0.02,"PASS",IF(AQ11&lt;0.04,"LEAN",IF(AQ11&lt;0.07,"SMALL",IF(AQ11&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ11&lt;=0,"PASS",IF(AQ11&lt;0.02,"PASS",IF(AQ11&lt;0.04,"LEAN",IF(AQ11&lt;0.07,"SMALL",IF(AQ11&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS11" s="4">
@@ -3587,7 +3587,7 @@
         <v/>
       </c>
       <c r="AW11">
-        <f>IF(AV11&lt;=0,"PASS",IF(AV11&lt;0.02,"PASS",IF(AV11&lt;0.04,"LEAN",IF(AV11&lt;0.07,"SMALL",IF(AV11&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV11&lt;=0,"PASS",IF(AV11&lt;0.02,"PASS",IF(AV11&lt;0.04,"LEAN",IF(AV11&lt;0.07,"SMALL",IF(AV11&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX11" s="4">
@@ -3607,7 +3607,7 @@
         <v/>
       </c>
       <c r="BB11">
-        <f>IF(BA11&lt;=0,"PASS",IF(BA11&lt;0.02,"PASS",IF(BA11&lt;0.04,"LEAN",IF(BA11&lt;0.07,"SMALL",IF(BA11&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA11&lt;=0,"PASS",IF(BA11&lt;0.02,"PASS",IF(BA11&lt;0.04,"LEAN",IF(BA11&lt;0.07,"SMALL",IF(BA11&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC11" s="4">
@@ -3834,7 +3834,7 @@
         <v/>
       </c>
       <c r="AR12">
-        <f>IF(AQ12&lt;=0,"PASS",IF(AQ12&lt;0.02,"PASS",IF(AQ12&lt;0.04,"LEAN",IF(AQ12&lt;0.07,"SMALL",IF(AQ12&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ12&lt;=0,"PASS",IF(AQ12&lt;0.02,"PASS",IF(AQ12&lt;0.04,"LEAN",IF(AQ12&lt;0.07,"SMALL",IF(AQ12&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS12" s="4">
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="AW12">
-        <f>IF(AV12&lt;=0,"PASS",IF(AV12&lt;0.02,"PASS",IF(AV12&lt;0.04,"LEAN",IF(AV12&lt;0.07,"SMALL",IF(AV12&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV12&lt;=0,"PASS",IF(AV12&lt;0.02,"PASS",IF(AV12&lt;0.04,"LEAN",IF(AV12&lt;0.07,"SMALL",IF(AV12&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX12" s="4">
@@ -3874,7 +3874,7 @@
         <v/>
       </c>
       <c r="BB12">
-        <f>IF(BA12&lt;=0,"PASS",IF(BA12&lt;0.02,"PASS",IF(BA12&lt;0.04,"LEAN",IF(BA12&lt;0.07,"SMALL",IF(BA12&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA12&lt;=0,"PASS",IF(BA12&lt;0.02,"PASS",IF(BA12&lt;0.04,"LEAN",IF(BA12&lt;0.07,"SMALL",IF(BA12&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC12" s="4">
@@ -4101,7 +4101,7 @@
         <v/>
       </c>
       <c r="AR13">
-        <f>IF(AQ13&lt;=0,"PASS",IF(AQ13&lt;0.02,"PASS",IF(AQ13&lt;0.04,"LEAN",IF(AQ13&lt;0.07,"SMALL",IF(AQ13&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ13&lt;=0,"PASS",IF(AQ13&lt;0.02,"PASS",IF(AQ13&lt;0.04,"LEAN",IF(AQ13&lt;0.07,"SMALL",IF(AQ13&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS13" s="4">
@@ -4121,7 +4121,7 @@
         <v/>
       </c>
       <c r="AW13">
-        <f>IF(AV13&lt;=0,"PASS",IF(AV13&lt;0.02,"PASS",IF(AV13&lt;0.04,"LEAN",IF(AV13&lt;0.07,"SMALL",IF(AV13&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV13&lt;=0,"PASS",IF(AV13&lt;0.02,"PASS",IF(AV13&lt;0.04,"LEAN",IF(AV13&lt;0.07,"SMALL",IF(AV13&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX13" s="4">
@@ -4141,7 +4141,7 @@
         <v/>
       </c>
       <c r="BB13">
-        <f>IF(BA13&lt;=0,"PASS",IF(BA13&lt;0.02,"PASS",IF(BA13&lt;0.04,"LEAN",IF(BA13&lt;0.07,"SMALL",IF(BA13&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA13&lt;=0,"PASS",IF(BA13&lt;0.02,"PASS",IF(BA13&lt;0.04,"LEAN",IF(BA13&lt;0.07,"SMALL",IF(BA13&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC13" s="4">
@@ -4368,7 +4368,7 @@
         <v/>
       </c>
       <c r="AR14">
-        <f>IF(AQ14&lt;=0,"PASS",IF(AQ14&lt;0.02,"PASS",IF(AQ14&lt;0.04,"LEAN",IF(AQ14&lt;0.07,"SMALL",IF(AQ14&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ14&lt;=0,"PASS",IF(AQ14&lt;0.02,"PASS",IF(AQ14&lt;0.04,"LEAN",IF(AQ14&lt;0.07,"SMALL",IF(AQ14&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS14" s="4">
@@ -4388,7 +4388,7 @@
         <v/>
       </c>
       <c r="AW14">
-        <f>IF(AV14&lt;=0,"PASS",IF(AV14&lt;0.02,"PASS",IF(AV14&lt;0.04,"LEAN",IF(AV14&lt;0.07,"SMALL",IF(AV14&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV14&lt;=0,"PASS",IF(AV14&lt;0.02,"PASS",IF(AV14&lt;0.04,"LEAN",IF(AV14&lt;0.07,"SMALL",IF(AV14&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX14" s="4">
@@ -4408,7 +4408,7 @@
         <v/>
       </c>
       <c r="BB14">
-        <f>IF(BA14&lt;=0,"PASS",IF(BA14&lt;0.02,"PASS",IF(BA14&lt;0.04,"LEAN",IF(BA14&lt;0.07,"SMALL",IF(BA14&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA14&lt;=0,"PASS",IF(BA14&lt;0.02,"PASS",IF(BA14&lt;0.04,"LEAN",IF(BA14&lt;0.07,"SMALL",IF(BA14&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC14" s="4">
@@ -4635,7 +4635,7 @@
         <v/>
       </c>
       <c r="AR15">
-        <f>IF(AQ15&lt;=0,"PASS",IF(AQ15&lt;0.02,"PASS",IF(AQ15&lt;0.04,"LEAN",IF(AQ15&lt;0.07,"SMALL",IF(AQ15&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ15&lt;=0,"PASS",IF(AQ15&lt;0.02,"PASS",IF(AQ15&lt;0.04,"LEAN",IF(AQ15&lt;0.07,"SMALL",IF(AQ15&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS15" s="4">
@@ -4655,7 +4655,7 @@
         <v/>
       </c>
       <c r="AW15">
-        <f>IF(AV15&lt;=0,"PASS",IF(AV15&lt;0.02,"PASS",IF(AV15&lt;0.04,"LEAN",IF(AV15&lt;0.07,"SMALL",IF(AV15&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV15&lt;=0,"PASS",IF(AV15&lt;0.02,"PASS",IF(AV15&lt;0.04,"LEAN",IF(AV15&lt;0.07,"SMALL",IF(AV15&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX15" s="4">
@@ -4675,7 +4675,7 @@
         <v/>
       </c>
       <c r="BB15">
-        <f>IF(BA15&lt;=0,"PASS",IF(BA15&lt;0.02,"PASS",IF(BA15&lt;0.04,"LEAN",IF(BA15&lt;0.07,"SMALL",IF(BA15&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA15&lt;=0,"PASS",IF(BA15&lt;0.02,"PASS",IF(BA15&lt;0.04,"LEAN",IF(BA15&lt;0.07,"SMALL",IF(BA15&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC15" s="4">
@@ -4902,7 +4902,7 @@
         <v/>
       </c>
       <c r="AR16">
-        <f>IF(AQ16&lt;=0,"PASS",IF(AQ16&lt;0.02,"PASS",IF(AQ16&lt;0.04,"LEAN",IF(AQ16&lt;0.07,"SMALL",IF(AQ16&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ16&lt;=0,"PASS",IF(AQ16&lt;0.02,"PASS",IF(AQ16&lt;0.04,"LEAN",IF(AQ16&lt;0.07,"SMALL",IF(AQ16&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS16" s="4">
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AW16">
-        <f>IF(AV16&lt;=0,"PASS",IF(AV16&lt;0.02,"PASS",IF(AV16&lt;0.04,"LEAN",IF(AV16&lt;0.07,"SMALL",IF(AV16&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV16&lt;=0,"PASS",IF(AV16&lt;0.02,"PASS",IF(AV16&lt;0.04,"LEAN",IF(AV16&lt;0.07,"SMALL",IF(AV16&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX16" s="4">
@@ -4942,7 +4942,7 @@
         <v/>
       </c>
       <c r="BB16">
-        <f>IF(BA16&lt;=0,"PASS",IF(BA16&lt;0.02,"PASS",IF(BA16&lt;0.04,"LEAN",IF(BA16&lt;0.07,"SMALL",IF(BA16&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA16&lt;=0,"PASS",IF(BA16&lt;0.02,"PASS",IF(BA16&lt;0.04,"LEAN",IF(BA16&lt;0.07,"SMALL",IF(BA16&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC16" s="4">
@@ -5169,7 +5169,7 @@
         <v/>
       </c>
       <c r="AR17">
-        <f>IF(AQ17&lt;=0,"PASS",IF(AQ17&lt;0.02,"PASS",IF(AQ17&lt;0.04,"LEAN",IF(AQ17&lt;0.07,"SMALL",IF(AQ17&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AQ17&lt;=0,"PASS",IF(AQ17&lt;0.02,"PASS",IF(AQ17&lt;0.04,"LEAN",IF(AQ17&lt;0.07,"SMALL",IF(AQ17&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AS17" s="4">
@@ -5189,7 +5189,7 @@
         <v/>
       </c>
       <c r="AW17">
-        <f>IF(AV17&lt;=0,"PASS",IF(AV17&lt;0.02,"PASS",IF(AV17&lt;0.04,"LEAN",IF(AV17&lt;0.07,"SMALL",IF(AV17&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AV17&lt;=0,"PASS",IF(AV17&lt;0.02,"PASS",IF(AV17&lt;0.04,"LEAN",IF(AV17&lt;0.07,"SMALL",IF(AV17&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AX17" s="4">
@@ -5209,7 +5209,7 @@
         <v/>
       </c>
       <c r="BB17">
-        <f>IF(BA17&lt;=0,"PASS",IF(BA17&lt;0.02,"PASS",IF(BA17&lt;0.04,"LEAN",IF(BA17&lt;0.07,"SMALL",IF(BA17&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(BA17&lt;=0,"PASS",IF(BA17&lt;0.02,"PASS",IF(BA17&lt;0.04,"LEAN",IF(BA17&lt;0.07,"SMALL",IF(BA17&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BC17" s="4">
@@ -5857,7 +5857,7 @@
         <v/>
       </c>
       <c r="AJ2">
-        <f>IF(AI2&lt;=0,"PASS",IF(AI2&lt;0.02,"PASS",IF(AI2&lt;0.04,"LEAN",IF(AI2&lt;0.07,"SMALL",IF(AI2&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI2&lt;=0,"PASS",IF(AI2&lt;0.02,"PASS",IF(AI2&lt;0.04,"LEAN",IF(AI2&lt;0.07,"SMALL",IF(AI2&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK2" s="4">
@@ -5877,7 +5877,7 @@
         <v/>
       </c>
       <c r="AO2">
-        <f>IF(AN2&lt;=0,"PASS",IF(AN2&lt;0.02,"PASS",IF(AN2&lt;0.04,"LEAN",IF(AN2&lt;0.07,"SMALL",IF(AN2&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN2&lt;=0,"PASS",IF(AN2&lt;0.02,"PASS",IF(AN2&lt;0.04,"LEAN",IF(AN2&lt;0.07,"SMALL",IF(AN2&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP2" s="4">
@@ -5921,7 +5921,7 @@
         <v/>
       </c>
       <c r="AZ2">
-        <f>IF(AY2&lt;=0,"PASS",IF(AY2&lt;0.02,"PASS",IF(AY2&lt;0.04,"LEAN",IF(AY2&lt;0.07,"SMALL",IF(AY2&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY2&lt;=0,"PASS",IF(AY2&lt;0.02,"PASS",IF(AY2&lt;0.04,"LEAN",IF(AY2&lt;0.07,"SMALL",IF(AY2&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA2" s="4">
@@ -6095,7 +6095,7 @@
         <v/>
       </c>
       <c r="AJ3">
-        <f>IF(AI3&lt;=0,"PASS",IF(AI3&lt;0.02,"PASS",IF(AI3&lt;0.04,"LEAN",IF(AI3&lt;0.07,"SMALL",IF(AI3&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI3&lt;=0,"PASS",IF(AI3&lt;0.02,"PASS",IF(AI3&lt;0.04,"LEAN",IF(AI3&lt;0.07,"SMALL",IF(AI3&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK3" s="4">
@@ -6115,7 +6115,7 @@
         <v/>
       </c>
       <c r="AO3">
-        <f>IF(AN3&lt;=0,"PASS",IF(AN3&lt;0.02,"PASS",IF(AN3&lt;0.04,"LEAN",IF(AN3&lt;0.07,"SMALL",IF(AN3&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN3&lt;=0,"PASS",IF(AN3&lt;0.02,"PASS",IF(AN3&lt;0.04,"LEAN",IF(AN3&lt;0.07,"SMALL",IF(AN3&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP3" s="4">
@@ -6159,7 +6159,7 @@
         <v/>
       </c>
       <c r="AZ3">
-        <f>IF(AY3&lt;=0,"PASS",IF(AY3&lt;0.02,"PASS",IF(AY3&lt;0.04,"LEAN",IF(AY3&lt;0.07,"SMALL",IF(AY3&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY3&lt;=0,"PASS",IF(AY3&lt;0.02,"PASS",IF(AY3&lt;0.04,"LEAN",IF(AY3&lt;0.07,"SMALL",IF(AY3&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA3" s="4">
@@ -6333,7 +6333,7 @@
         <v/>
       </c>
       <c r="AJ4">
-        <f>IF(AI4&lt;=0,"PASS",IF(AI4&lt;0.02,"PASS",IF(AI4&lt;0.04,"LEAN",IF(AI4&lt;0.07,"SMALL",IF(AI4&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI4&lt;=0,"PASS",IF(AI4&lt;0.02,"PASS",IF(AI4&lt;0.04,"LEAN",IF(AI4&lt;0.07,"SMALL",IF(AI4&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK4" s="4">
@@ -6353,7 +6353,7 @@
         <v/>
       </c>
       <c r="AO4">
-        <f>IF(AN4&lt;=0,"PASS",IF(AN4&lt;0.02,"PASS",IF(AN4&lt;0.04,"LEAN",IF(AN4&lt;0.07,"SMALL",IF(AN4&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN4&lt;=0,"PASS",IF(AN4&lt;0.02,"PASS",IF(AN4&lt;0.04,"LEAN",IF(AN4&lt;0.07,"SMALL",IF(AN4&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP4" s="4">
@@ -6397,7 +6397,7 @@
         <v/>
       </c>
       <c r="AZ4">
-        <f>IF(AY4&lt;=0,"PASS",IF(AY4&lt;0.02,"PASS",IF(AY4&lt;0.04,"LEAN",IF(AY4&lt;0.07,"SMALL",IF(AY4&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY4&lt;=0,"PASS",IF(AY4&lt;0.02,"PASS",IF(AY4&lt;0.04,"LEAN",IF(AY4&lt;0.07,"SMALL",IF(AY4&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA4" s="4">
@@ -6571,7 +6571,7 @@
         <v/>
       </c>
       <c r="AJ5">
-        <f>IF(AI5&lt;=0,"PASS",IF(AI5&lt;0.02,"PASS",IF(AI5&lt;0.04,"LEAN",IF(AI5&lt;0.07,"SMALL",IF(AI5&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI5&lt;=0,"PASS",IF(AI5&lt;0.02,"PASS",IF(AI5&lt;0.04,"LEAN",IF(AI5&lt;0.07,"SMALL",IF(AI5&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK5" s="4">
@@ -6591,7 +6591,7 @@
         <v/>
       </c>
       <c r="AO5">
-        <f>IF(AN5&lt;=0,"PASS",IF(AN5&lt;0.02,"PASS",IF(AN5&lt;0.04,"LEAN",IF(AN5&lt;0.07,"SMALL",IF(AN5&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN5&lt;=0,"PASS",IF(AN5&lt;0.02,"PASS",IF(AN5&lt;0.04,"LEAN",IF(AN5&lt;0.07,"SMALL",IF(AN5&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP5" s="4">
@@ -6635,7 +6635,7 @@
         <v/>
       </c>
       <c r="AZ5">
-        <f>IF(AY5&lt;=0,"PASS",IF(AY5&lt;0.02,"PASS",IF(AY5&lt;0.04,"LEAN",IF(AY5&lt;0.07,"SMALL",IF(AY5&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY5&lt;=0,"PASS",IF(AY5&lt;0.02,"PASS",IF(AY5&lt;0.04,"LEAN",IF(AY5&lt;0.07,"SMALL",IF(AY5&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA5" s="4">
@@ -6809,7 +6809,7 @@
         <v/>
       </c>
       <c r="AJ6">
-        <f>IF(AI6&lt;=0,"PASS",IF(AI6&lt;0.02,"PASS",IF(AI6&lt;0.04,"LEAN",IF(AI6&lt;0.07,"SMALL",IF(AI6&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI6&lt;=0,"PASS",IF(AI6&lt;0.02,"PASS",IF(AI6&lt;0.04,"LEAN",IF(AI6&lt;0.07,"SMALL",IF(AI6&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK6" s="4">
@@ -6829,7 +6829,7 @@
         <v/>
       </c>
       <c r="AO6">
-        <f>IF(AN6&lt;=0,"PASS",IF(AN6&lt;0.02,"PASS",IF(AN6&lt;0.04,"LEAN",IF(AN6&lt;0.07,"SMALL",IF(AN6&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN6&lt;=0,"PASS",IF(AN6&lt;0.02,"PASS",IF(AN6&lt;0.04,"LEAN",IF(AN6&lt;0.07,"SMALL",IF(AN6&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP6" s="4">
@@ -6873,7 +6873,7 @@
         <v/>
       </c>
       <c r="AZ6">
-        <f>IF(AY6&lt;=0,"PASS",IF(AY6&lt;0.02,"PASS",IF(AY6&lt;0.04,"LEAN",IF(AY6&lt;0.07,"SMALL",IF(AY6&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY6&lt;=0,"PASS",IF(AY6&lt;0.02,"PASS",IF(AY6&lt;0.04,"LEAN",IF(AY6&lt;0.07,"SMALL",IF(AY6&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA6" s="4">
@@ -7047,7 +7047,7 @@
         <v/>
       </c>
       <c r="AJ7">
-        <f>IF(AI7&lt;=0,"PASS",IF(AI7&lt;0.02,"PASS",IF(AI7&lt;0.04,"LEAN",IF(AI7&lt;0.07,"SMALL",IF(AI7&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI7&lt;=0,"PASS",IF(AI7&lt;0.02,"PASS",IF(AI7&lt;0.04,"LEAN",IF(AI7&lt;0.07,"SMALL",IF(AI7&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK7" s="4">
@@ -7067,7 +7067,7 @@
         <v/>
       </c>
       <c r="AO7">
-        <f>IF(AN7&lt;=0,"PASS",IF(AN7&lt;0.02,"PASS",IF(AN7&lt;0.04,"LEAN",IF(AN7&lt;0.07,"SMALL",IF(AN7&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN7&lt;=0,"PASS",IF(AN7&lt;0.02,"PASS",IF(AN7&lt;0.04,"LEAN",IF(AN7&lt;0.07,"SMALL",IF(AN7&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP7" s="4">
@@ -7111,7 +7111,7 @@
         <v/>
       </c>
       <c r="AZ7">
-        <f>IF(AY7&lt;=0,"PASS",IF(AY7&lt;0.02,"PASS",IF(AY7&lt;0.04,"LEAN",IF(AY7&lt;0.07,"SMALL",IF(AY7&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY7&lt;=0,"PASS",IF(AY7&lt;0.02,"PASS",IF(AY7&lt;0.04,"LEAN",IF(AY7&lt;0.07,"SMALL",IF(AY7&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA7" s="4">
@@ -7285,7 +7285,7 @@
         <v/>
       </c>
       <c r="AJ8">
-        <f>IF(AI8&lt;=0,"PASS",IF(AI8&lt;0.02,"PASS",IF(AI8&lt;0.04,"LEAN",IF(AI8&lt;0.07,"SMALL",IF(AI8&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI8&lt;=0,"PASS",IF(AI8&lt;0.02,"PASS",IF(AI8&lt;0.04,"LEAN",IF(AI8&lt;0.07,"SMALL",IF(AI8&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK8" s="4">
@@ -7305,7 +7305,7 @@
         <v/>
       </c>
       <c r="AO8">
-        <f>IF(AN8&lt;=0,"PASS",IF(AN8&lt;0.02,"PASS",IF(AN8&lt;0.04,"LEAN",IF(AN8&lt;0.07,"SMALL",IF(AN8&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN8&lt;=0,"PASS",IF(AN8&lt;0.02,"PASS",IF(AN8&lt;0.04,"LEAN",IF(AN8&lt;0.07,"SMALL",IF(AN8&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP8" s="4">
@@ -7349,7 +7349,7 @@
         <v/>
       </c>
       <c r="AZ8">
-        <f>IF(AY8&lt;=0,"PASS",IF(AY8&lt;0.02,"PASS",IF(AY8&lt;0.04,"LEAN",IF(AY8&lt;0.07,"SMALL",IF(AY8&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY8&lt;=0,"PASS",IF(AY8&lt;0.02,"PASS",IF(AY8&lt;0.04,"LEAN",IF(AY8&lt;0.07,"SMALL",IF(AY8&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA8" s="4">
@@ -7523,7 +7523,7 @@
         <v/>
       </c>
       <c r="AJ9">
-        <f>IF(AI9&lt;=0,"PASS",IF(AI9&lt;0.02,"PASS",IF(AI9&lt;0.04,"LEAN",IF(AI9&lt;0.07,"SMALL",IF(AI9&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI9&lt;=0,"PASS",IF(AI9&lt;0.02,"PASS",IF(AI9&lt;0.04,"LEAN",IF(AI9&lt;0.07,"SMALL",IF(AI9&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK9" s="4">
@@ -7543,7 +7543,7 @@
         <v/>
       </c>
       <c r="AO9">
-        <f>IF(AN9&lt;=0,"PASS",IF(AN9&lt;0.02,"PASS",IF(AN9&lt;0.04,"LEAN",IF(AN9&lt;0.07,"SMALL",IF(AN9&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN9&lt;=0,"PASS",IF(AN9&lt;0.02,"PASS",IF(AN9&lt;0.04,"LEAN",IF(AN9&lt;0.07,"SMALL",IF(AN9&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP9" s="4">
@@ -7587,7 +7587,7 @@
         <v/>
       </c>
       <c r="AZ9">
-        <f>IF(AY9&lt;=0,"PASS",IF(AY9&lt;0.02,"PASS",IF(AY9&lt;0.04,"LEAN",IF(AY9&lt;0.07,"SMALL",IF(AY9&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY9&lt;=0,"PASS",IF(AY9&lt;0.02,"PASS",IF(AY9&lt;0.04,"LEAN",IF(AY9&lt;0.07,"SMALL",IF(AY9&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA9" s="4">
@@ -7761,7 +7761,7 @@
         <v/>
       </c>
       <c r="AJ10">
-        <f>IF(AI10&lt;=0,"PASS",IF(AI10&lt;0.02,"PASS",IF(AI10&lt;0.04,"LEAN",IF(AI10&lt;0.07,"SMALL",IF(AI10&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI10&lt;=0,"PASS",IF(AI10&lt;0.02,"PASS",IF(AI10&lt;0.04,"LEAN",IF(AI10&lt;0.07,"SMALL",IF(AI10&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK10" s="4">
@@ -7781,7 +7781,7 @@
         <v/>
       </c>
       <c r="AO10">
-        <f>IF(AN10&lt;=0,"PASS",IF(AN10&lt;0.02,"PASS",IF(AN10&lt;0.04,"LEAN",IF(AN10&lt;0.07,"SMALL",IF(AN10&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN10&lt;=0,"PASS",IF(AN10&lt;0.02,"PASS",IF(AN10&lt;0.04,"LEAN",IF(AN10&lt;0.07,"SMALL",IF(AN10&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP10" s="4">
@@ -7825,7 +7825,7 @@
         <v/>
       </c>
       <c r="AZ10">
-        <f>IF(AY10&lt;=0,"PASS",IF(AY10&lt;0.02,"PASS",IF(AY10&lt;0.04,"LEAN",IF(AY10&lt;0.07,"SMALL",IF(AY10&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY10&lt;=0,"PASS",IF(AY10&lt;0.02,"PASS",IF(AY10&lt;0.04,"LEAN",IF(AY10&lt;0.07,"SMALL",IF(AY10&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA10" s="4">
@@ -7999,7 +7999,7 @@
         <v/>
       </c>
       <c r="AJ11">
-        <f>IF(AI11&lt;=0,"PASS",IF(AI11&lt;0.02,"PASS",IF(AI11&lt;0.04,"LEAN",IF(AI11&lt;0.07,"SMALL",IF(AI11&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI11&lt;=0,"PASS",IF(AI11&lt;0.02,"PASS",IF(AI11&lt;0.04,"LEAN",IF(AI11&lt;0.07,"SMALL",IF(AI11&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK11" s="4">
@@ -8019,7 +8019,7 @@
         <v/>
       </c>
       <c r="AO11">
-        <f>IF(AN11&lt;=0,"PASS",IF(AN11&lt;0.02,"PASS",IF(AN11&lt;0.04,"LEAN",IF(AN11&lt;0.07,"SMALL",IF(AN11&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN11&lt;=0,"PASS",IF(AN11&lt;0.02,"PASS",IF(AN11&lt;0.04,"LEAN",IF(AN11&lt;0.07,"SMALL",IF(AN11&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP11" s="4">
@@ -8063,7 +8063,7 @@
         <v/>
       </c>
       <c r="AZ11">
-        <f>IF(AY11&lt;=0,"PASS",IF(AY11&lt;0.02,"PASS",IF(AY11&lt;0.04,"LEAN",IF(AY11&lt;0.07,"SMALL",IF(AY11&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY11&lt;=0,"PASS",IF(AY11&lt;0.02,"PASS",IF(AY11&lt;0.04,"LEAN",IF(AY11&lt;0.07,"SMALL",IF(AY11&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA11" s="4">
@@ -8237,7 +8237,7 @@
         <v/>
       </c>
       <c r="AJ12">
-        <f>IF(AI12&lt;=0,"PASS",IF(AI12&lt;0.02,"PASS",IF(AI12&lt;0.04,"LEAN",IF(AI12&lt;0.07,"SMALL",IF(AI12&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI12&lt;=0,"PASS",IF(AI12&lt;0.02,"PASS",IF(AI12&lt;0.04,"LEAN",IF(AI12&lt;0.07,"SMALL",IF(AI12&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK12" s="4">
@@ -8257,7 +8257,7 @@
         <v/>
       </c>
       <c r="AO12">
-        <f>IF(AN12&lt;=0,"PASS",IF(AN12&lt;0.02,"PASS",IF(AN12&lt;0.04,"LEAN",IF(AN12&lt;0.07,"SMALL",IF(AN12&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN12&lt;=0,"PASS",IF(AN12&lt;0.02,"PASS",IF(AN12&lt;0.04,"LEAN",IF(AN12&lt;0.07,"SMALL",IF(AN12&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP12" s="4">
@@ -8301,7 +8301,7 @@
         <v/>
       </c>
       <c r="AZ12">
-        <f>IF(AY12&lt;=0,"PASS",IF(AY12&lt;0.02,"PASS",IF(AY12&lt;0.04,"LEAN",IF(AY12&lt;0.07,"SMALL",IF(AY12&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY12&lt;=0,"PASS",IF(AY12&lt;0.02,"PASS",IF(AY12&lt;0.04,"LEAN",IF(AY12&lt;0.07,"SMALL",IF(AY12&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA12" s="4">
@@ -8475,7 +8475,7 @@
         <v/>
       </c>
       <c r="AJ13">
-        <f>IF(AI13&lt;=0,"PASS",IF(AI13&lt;0.02,"PASS",IF(AI13&lt;0.04,"LEAN",IF(AI13&lt;0.07,"SMALL",IF(AI13&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI13&lt;=0,"PASS",IF(AI13&lt;0.02,"PASS",IF(AI13&lt;0.04,"LEAN",IF(AI13&lt;0.07,"SMALL",IF(AI13&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK13" s="4">
@@ -8495,7 +8495,7 @@
         <v/>
       </c>
       <c r="AO13">
-        <f>IF(AN13&lt;=0,"PASS",IF(AN13&lt;0.02,"PASS",IF(AN13&lt;0.04,"LEAN",IF(AN13&lt;0.07,"SMALL",IF(AN13&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN13&lt;=0,"PASS",IF(AN13&lt;0.02,"PASS",IF(AN13&lt;0.04,"LEAN",IF(AN13&lt;0.07,"SMALL",IF(AN13&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP13" s="4">
@@ -8539,7 +8539,7 @@
         <v/>
       </c>
       <c r="AZ13">
-        <f>IF(AY13&lt;=0,"PASS",IF(AY13&lt;0.02,"PASS",IF(AY13&lt;0.04,"LEAN",IF(AY13&lt;0.07,"SMALL",IF(AY13&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY13&lt;=0,"PASS",IF(AY13&lt;0.02,"PASS",IF(AY13&lt;0.04,"LEAN",IF(AY13&lt;0.07,"SMALL",IF(AY13&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA13" s="4">
@@ -8713,7 +8713,7 @@
         <v/>
       </c>
       <c r="AJ14">
-        <f>IF(AI14&lt;=0,"PASS",IF(AI14&lt;0.02,"PASS",IF(AI14&lt;0.04,"LEAN",IF(AI14&lt;0.07,"SMALL",IF(AI14&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI14&lt;=0,"PASS",IF(AI14&lt;0.02,"PASS",IF(AI14&lt;0.04,"LEAN",IF(AI14&lt;0.07,"SMALL",IF(AI14&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK14" s="4">
@@ -8733,7 +8733,7 @@
         <v/>
       </c>
       <c r="AO14">
-        <f>IF(AN14&lt;=0,"PASS",IF(AN14&lt;0.02,"PASS",IF(AN14&lt;0.04,"LEAN",IF(AN14&lt;0.07,"SMALL",IF(AN14&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN14&lt;=0,"PASS",IF(AN14&lt;0.02,"PASS",IF(AN14&lt;0.04,"LEAN",IF(AN14&lt;0.07,"SMALL",IF(AN14&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP14" s="4">
@@ -8777,7 +8777,7 @@
         <v/>
       </c>
       <c r="AZ14">
-        <f>IF(AY14&lt;=0,"PASS",IF(AY14&lt;0.02,"PASS",IF(AY14&lt;0.04,"LEAN",IF(AY14&lt;0.07,"SMALL",IF(AY14&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY14&lt;=0,"PASS",IF(AY14&lt;0.02,"PASS",IF(AY14&lt;0.04,"LEAN",IF(AY14&lt;0.07,"SMALL",IF(AY14&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA14" s="4">
@@ -8951,7 +8951,7 @@
         <v/>
       </c>
       <c r="AJ15">
-        <f>IF(AI15&lt;=0,"PASS",IF(AI15&lt;0.02,"PASS",IF(AI15&lt;0.04,"LEAN",IF(AI15&lt;0.07,"SMALL",IF(AI15&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI15&lt;=0,"PASS",IF(AI15&lt;0.02,"PASS",IF(AI15&lt;0.04,"LEAN",IF(AI15&lt;0.07,"SMALL",IF(AI15&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK15" s="4">
@@ -8971,7 +8971,7 @@
         <v/>
       </c>
       <c r="AO15">
-        <f>IF(AN15&lt;=0,"PASS",IF(AN15&lt;0.02,"PASS",IF(AN15&lt;0.04,"LEAN",IF(AN15&lt;0.07,"SMALL",IF(AN15&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN15&lt;=0,"PASS",IF(AN15&lt;0.02,"PASS",IF(AN15&lt;0.04,"LEAN",IF(AN15&lt;0.07,"SMALL",IF(AN15&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP15" s="4">
@@ -9015,7 +9015,7 @@
         <v/>
       </c>
       <c r="AZ15">
-        <f>IF(AY15&lt;=0,"PASS",IF(AY15&lt;0.02,"PASS",IF(AY15&lt;0.04,"LEAN",IF(AY15&lt;0.07,"SMALL",IF(AY15&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY15&lt;=0,"PASS",IF(AY15&lt;0.02,"PASS",IF(AY15&lt;0.04,"LEAN",IF(AY15&lt;0.07,"SMALL",IF(AY15&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA15" s="4">
@@ -9189,7 +9189,7 @@
         <v/>
       </c>
       <c r="AJ16">
-        <f>IF(AI16&lt;=0,"PASS",IF(AI16&lt;0.02,"PASS",IF(AI16&lt;0.04,"LEAN",IF(AI16&lt;0.07,"SMALL",IF(AI16&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI16&lt;=0,"PASS",IF(AI16&lt;0.02,"PASS",IF(AI16&lt;0.04,"LEAN",IF(AI16&lt;0.07,"SMALL",IF(AI16&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK16" s="4">
@@ -9209,7 +9209,7 @@
         <v/>
       </c>
       <c r="AO16">
-        <f>IF(AN16&lt;=0,"PASS",IF(AN16&lt;0.02,"PASS",IF(AN16&lt;0.04,"LEAN",IF(AN16&lt;0.07,"SMALL",IF(AN16&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN16&lt;=0,"PASS",IF(AN16&lt;0.02,"PASS",IF(AN16&lt;0.04,"LEAN",IF(AN16&lt;0.07,"SMALL",IF(AN16&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP16" s="4">
@@ -9253,7 +9253,7 @@
         <v/>
       </c>
       <c r="AZ16">
-        <f>IF(AY16&lt;=0,"PASS",IF(AY16&lt;0.02,"PASS",IF(AY16&lt;0.04,"LEAN",IF(AY16&lt;0.07,"SMALL",IF(AY16&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY16&lt;=0,"PASS",IF(AY16&lt;0.02,"PASS",IF(AY16&lt;0.04,"LEAN",IF(AY16&lt;0.07,"SMALL",IF(AY16&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA16" s="4">
@@ -9427,7 +9427,7 @@
         <v/>
       </c>
       <c r="AJ17">
-        <f>IF(AI17&lt;=0,"PASS",IF(AI17&lt;0.02,"PASS",IF(AI17&lt;0.04,"LEAN",IF(AI17&lt;0.07,"SMALL",IF(AI17&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AI17&lt;=0,"PASS",IF(AI17&lt;0.02,"PASS",IF(AI17&lt;0.04,"LEAN",IF(AI17&lt;0.07,"SMALL",IF(AI17&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AK17" s="4">
@@ -9447,7 +9447,7 @@
         <v/>
       </c>
       <c r="AO17">
-        <f>IF(AN17&lt;=0,"PASS",IF(AN17&lt;0.02,"PASS",IF(AN17&lt;0.04,"LEAN",IF(AN17&lt;0.07,"SMALL",IF(AN17&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AN17&lt;=0,"PASS",IF(AN17&lt;0.02,"PASS",IF(AN17&lt;0.04,"LEAN",IF(AN17&lt;0.07,"SMALL",IF(AN17&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="AP17" s="4">
@@ -9491,7 +9491,7 @@
         <v/>
       </c>
       <c r="AZ17">
-        <f>IF(AY17&lt;=0,"PASS",IF(AY17&lt;0.02,"PASS",IF(AY17&lt;0.04,"LEAN",IF(AY17&lt;0.07,"SMALL",IF(AY17&lt;0.10,"MEDIUM","STRONG"))))))</f>
+        <f>IF(AY17&lt;=0,"PASS",IF(AY17&lt;0.02,"PASS",IF(AY17&lt;0.04,"LEAN",IF(AY17&lt;0.07,"SMALL",IF(AY17&lt;0.10,"MEDIUM","STRONG")))))</f>
         <v/>
       </c>
       <c r="BA17" s="4">

</xml_diff>